<commit_message>
docs(enterprise): advance snapshot after branch rebase
</commit_message>
<xml_diff>
--- a/smartlock-docs/enterprise/規格統控整理/SmartLock_規格統控規劃書.xlsx
+++ b/smartlock-docs/enterprise/規格統控整理/SmartLock_規格統控規劃書.xlsx
@@ -1395,7 +1395,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>🔶 drift-check ✅ 2026-07-09（CR-0136：migration 檔案層守門 CI＋12 支波次補登；Cloud Run CD 觸發器＝OPS）</t>
+          <t>🔶 drift-check ✅ 2026-07-09（CR-0136：migration 檔案層守門 CI＋12 支波次補登；Cloud Run CD 觸發器＝OPS）〔標注 2026-07-27：再增兩道 CI gate——①web-lint-typecheck.yml（四站 matrix tsc+eslint；補前發現四站 npm run lint 因無 ESLint 設定與依賴而從未運作過）②scripts/ci/endpoint-guard-audit.py（端點守衛不對稱雙檢：v2/legacy 孿生＋list/detail），已反向驗證有效（修復前抓 8 組、修復後清零）〕</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>✅ 2026-07-09（CR-0137：api 1719 passed 全綠＋修 seed 順序 bug/測試污染/legacy 斷言；1 live 測試 Vertex 429 非迴歸）</t>
+          <t>✅ 2026-07-09（CR-0137：api 1719 passed 全綠＋修 seed 順序 bug/測試污染/legacy 斷言；1 live 測試 Vertex 429 非迴歸）〔標注 2026-07-27：全套回歸能力解封——新增 scripts/db/make-test-db.sh（pg_dump 複製 UAT 庫＋補套 migration 建隔離 scratch 庫），此前因 pytest 單庫 fallback 直打 5433 UAT 庫而無法安全跑全套。實測 api 2091 passed / 13 failed（13 支 seed 依賴非回歸）＋agent 309 passed；並據此確認本輪 20 個端點角色守衛變更零回歸〕</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat(plane): 敏捷每週衝刺——sprint_plan.yaml 宣告 + 規劃書 ④ + Plane cycles
四書原本沒有任何排程載體：③ 回答「有哪些工作」，但「哪一週做」無處可放。
而 cycle 是這個平台唯一會自動產圖的地方（burndown）——沒有它，「這個節點
會不會滑」就只剩人每週口頭回報，而口頭回報一向是最樂觀的那個版本。

排程是宣告不是推導：前置依賴只給得出「不能早於」，給不出「應該在哪一週」，
那是人衡量產能、風險與承諾後的決定。所以 sprint_plan.yaml 與四條邊同性質
（人宣告、不可推導）但不是邊——不進 _validate_relations.py，不影響追溯。
_relations/ 現有兩個這類非邊檔，指南 §4 改成表格明列以免被當成第五條邊。

範圍砍過而且指名：24 個未完成工作包中，M4 的 7 項屬階段二（flow DSL 引擎、
FlowEditor、AI Onboarding Compiler、第 2 產業落地…），全在 Backlog、無前置、
無排程，五週做不完，列 out_of_scope 並在分頁上以紅字 banner 指名；3.1.3 混合
派工卡在 CR-0191 §8 六項裁決，列 blocked。不指名的代價是期末沒做完會被讀成
滑期，而它從一開始就不在範圍內。實排 16 張進 S1–S5（07-27 ~ 08-31）。

另記：Sprint 1 只剩四個工作天（指示下達日 07-29 是週三），這不是估錯是起跑點
就在週中，先寫下來免得第一週未達標被當成速度問題。

踩到 Cycle.description 是純字串 TextField 而 TestRun.description 是
{"text": ...} JSON——同名欄位在兩個模型不同形狀，套錯直接 400。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TkrnDv8YDbyRz7ZRzN69ah
</commit_message>
<xml_diff>
--- a/smartlock-docs/enterprise/規格統控整理/SmartLock_規格統控規劃書.xlsx
+++ b/smartlock-docs/enterprise/規格統控整理/SmartLock_規格統控規劃書.xlsx
@@ -10,10 +10,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="① 怎麼用這本" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="② 缺口與決策清單" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="③ 里程碑與已定案決策" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="④ 迭代計畫（每週衝刺）" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'② 缺口與決策清單'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'③ 里程碑與已定案決策'!$A$1:$G$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'④ 迭代計畫（每週衝刺）'!$A$1:$K$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -107,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -131,6 +133,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -498,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -577,145 +582,169 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="1" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>③ 與 ④ 差在哪</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>③ 回答「有哪些工作」，④ 回答「哪一週做」。排程算不出來——前置依賴只給得出「不能早於」，給不出「應該在哪一週」，所以 ④ 的來源是宣告檔 _relations/sprint_plan.yaml，一列一個決定。</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
+          <t>④ 底下那兩段紅字要看</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>「待裁決」是卡在人身上、不是卡在工程；「明確排除」是範圍砍掉的決定。兩者都刻意指名——不指名的話，期末沒做完會被讀成滑期，而它從一開始就不在範圍內。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="1" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
           <t>Plane 詞彙對照</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>本書的列在 Plane 專案管理系統裡叫什麼（依《Plane QA 工程守則》Part B）。跨系統討論一律用右欄的名字——同一件事兩個名字，是對帳失敗最常見的起點。</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  里程碑 M1–M5</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Plane 的 Milestone（Issue.milestone，單值，所以一張卡只能掛一個節點）。</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  階段一 / 階段二</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Plane 的 Initiative（workspace 級，掛專案而非掛卡）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  WBS 工作包</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Plane 的 Task（level 3）。它有負責人與前置依賴、用技術語彙，是交付物分解不是價值切片——不要為了湊 Story 層把它改寫成「作為…我想要…」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  本表的缺口 ≠ 出貨閘門的 blocker</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>本表 ② 是「規格側」的追溯缺口（V2/V7/V8/V9/V10，設計有沒有接好）；Plane 出貨閘門的 blocker 是「執行側」的五類（failed／blocked／未結缺陷／未執行／已排程卻零契約）。兩套各自成立、不得互推——設計全綠不代表跑得過，反之亦然。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">  WBS 工作包</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Plane 的 Task（level 3）。它有負責人與前置依賴、用技術語彙，是交付物分解不是價值切片——不要為了湊 Story 層把它改寫成「作為…我想要…」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  本表的缺口 ≠ 出貨閘門的 blocker</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>本表 ② 是「規格側」的追溯缺口（V2/V7/V8/V9/V10，設計有沒有接好）；Plane 出貨閘門的 blocker 是「執行側」的五類（failed／blocked／未結缺陷／未執行／已排程卻零契約）。兩套各自成立、不得互推——設計全綠不代表跑得過，反之亦然。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">  本專案目前沒有 Cycle</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Plane 的 Cycle 是迭代時間盒。本專案的排程只到 Milestone 層，尚未建任何 cycle；在那之前「這個 sprint 交付什麼」這個問題沒有載體。</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="1" t="inlineStr"/>
-      <c r="B14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>黃色欄位</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>只有人能填。系統不會、也不該幫你填。</t>
-        </is>
-      </c>
-    </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>灰色欄位</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>生成欄，手改會在下次重跑被覆蓋。要改請改上游 Markdown 或 _relations/*.yaml。</t>
-        </is>
-      </c>
+      <c r="A16" s="1" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
+          <t>黃色欄位</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>只有人能填。系統不會、也不該幫你填。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>灰色欄位</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>生成欄，手改會在下次重跑被覆蓋。要改請改上游 Markdown 或 _relations/*.yaml。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
           <t>白色欄位</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>正典敘述，同樣改上游。</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="1" t="inlineStr"/>
-      <c r="B18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="1" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>四個狀態軸不得互推</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>程式檔存在 ≠ 工程完成；工程完成 ≠ 測試通過；測試通過 ≠ 驗收通過。需求定版(SA) / 工程證據(RD) / 測試執行(QA) / 驗收通過(業務 Owner) 各有唯一 owner，任何一格都不得由另一軸自動帶出。</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>怎麼重生</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>改上游正典 → 在 規格統控整理/ 跑 python3 _build_workbooks.py。xlsx 是單向快照，永遠不要直接改 xlsx 再往回抄。</t>
         </is>
@@ -4251,4 +4280,1187 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>衝刺</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>期間</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>衝刺目標</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>WBS</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>工作包</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>目前狀態</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>前置</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>本衝刺完成？</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>實際完成日</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-27 ~ 2026-08-02</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>可觀測性與 CD 兩條 M1 尾巴收乾淨，讓 M2 的前置條件成立</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>1.4.1</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>可觀測性：SigNoz（metrics/logs/traces/alerts）+ OPIK（LLM 品質）基線</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>🔶 code 面 ✅（CR-0136 api＋CR-0156 agent/ref</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr"/>
+      <c r="J2" s="8" t="inlineStr"/>
+      <c r="K2" s="8" t="inlineStr"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-27 ~ 2026-08-02</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>可觀測性與 CD 兩條 M1 尾巴收乾淨，讓 M2 的前置條件成立</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>基礎 CD：3 Cloud Run 自動部署 + migration drift-check CI</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>🔶 drift-check ✅ 2026-07-09（CR-0136：migra</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr"/>
+      <c r="J3" s="8" t="inlineStr"/>
+      <c r="K3" s="8" t="inlineStr"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03 ~ 2026-08-09</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Casdoor 統一 IdP、技師平台獨立、v1 API 收斂三線並行</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>2.1.1</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Casdoor 統一 IdP：org（租戶）/ OIDC 授權碼流 / License 訂閱管理</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>🔶 R1 ✅ 2026-07-10（CR-0141：Casdoor 部署 pro</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr"/>
+      <c r="J4" s="8" t="inlineStr"/>
+      <c r="K4" s="8" t="inlineStr"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03 ~ 2026-08-09</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Casdoor 統一 IdP、技師平台獨立、v1 API 收斂三線並行</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>2.4.1</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>technician-platform 獨立系統：技師庫 + tech-api + 師傅 web 拆出</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>🔶 方案A/B 已落地（CR-0112：雙 stack＋技師身分權威庫拆分＋投影</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr"/>
+      <c r="J5" s="8" t="inlineStr"/>
+      <c r="K5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03 ~ 2026-08-09</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Casdoor 統一 IdP、技師平台獨立、v1 API 收斂三線並行</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>2.5.1</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>v1 API 收斂：凍結 → 遷移 ~42 caller → 移除（5-gate）</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>🔶 Gate-1 凍結 enforced 2026-07-10（CR-0145：</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr"/>
+      <c r="J6" s="8" t="inlineStr"/>
+      <c r="K6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-10 ~ 2026-08-16</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>M2 SIT+UAT 通過；憑證生命週期與背景 runtime 拆分落地</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>2.6.1</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>M2 SIT + UAT（含跨系統整合場景）</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>🔶 SIT ✅ 2026-07-10（CR-0147：api 1738＋agen</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>2.1–2.5</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr"/>
+      <c r="J7" s="8" t="inlineStr"/>
+      <c r="K7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-10 ~ 2026-08-16</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>M2 SIT+UAT 通過；憑證生命週期與背景 runtime 拆分落地</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>3.6.5</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>M3.6</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Service principal／credential lifecycle：hash、scope、expiry、rotation、revoke、audit；遷移共用 X-Internal-Token</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>🟨 code ready／待 production gate</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>ADR-036；ADR-040／ADR-041（OD-001／004 已 closed）</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr"/>
+      <c r="J8" s="8" t="inlineStr"/>
+      <c r="K8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-10 ~ 2026-08-16</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>M2 SIT+UAT 通過；憑證生命週期與背景 runtime 拆分落地</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>3.6.6</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>M3.6</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Background runtime 拆分：job registry、worker entrypoint、Cloud Scheduler/Run Job pilot、outbox metrics</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>🟨 pilot ready／待 GCP 演練</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>ADR-037；GCP IAM/Scheduler</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr"/>
+      <c r="J9" s="8" t="inlineStr"/>
+      <c r="K9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-17 ~ 2026-08-23</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Kafka 事件骨幹上線；License → provisioning 自動化；promotion 流程定版</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Kafka 事件骨幹：commission.accrued / 工單投影事件上線（替換 outbox 輪詢）</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>⬜〔標注 2026-07-22（Plane 對帳輪）：Plane 卡=In Pr</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>階段閘</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr"/>
+      <c r="J10" s="8" t="inlineStr"/>
+      <c r="K10" s="8" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-17 ~ 2026-08-23</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Kafka 事件骨幹上線；License → provisioning 自動化；promotion 流程定版</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>3.3.1</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>License → provisioning 自動化（開站流程腳本化）</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>⬜〔標注 2026-07-28：ADR-042 生效後，開站不再需要為 refi</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>2.1.1</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr"/>
+      <c r="J11" s="8" t="inlineStr"/>
+      <c r="K11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-17 ~ 2026-08-23</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Kafka 事件骨幹上線；License → provisioning 自動化；promotion 流程定版</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>3.6.7</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>M3.6</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>GCP staging→production promotion、GitHub Environments、WIF 隔離、release manifest、rollback/restore evidence</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>🟨 workflow ready／待外部環境</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>ADR-038；3.6.4；3.6.6</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr"/>
+      <c r="J12" s="8" t="inlineStr"/>
+      <c r="K12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-24 ~ 2026-08-31</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>投影、對帳、intake 契約與第 2 品牌開站演練，M3 收斂</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>3.1.2</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>技師工作台改吃 CQRS 投影（跨品牌工單聚合）</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⬜〔標注 2026-07-28：ADR-043 已定版師傅專屬 channel </t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>3.1.1 / 2.4.1</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr"/>
+      <c r="J13" s="8" t="inlineStr"/>
+      <c r="K13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-24 ~ 2026-08-31</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>投影、對帳、intake 契約與第 2 品牌開站演練，M3 收斂</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>3.2.1</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>期末對帳 reconcile 閘門（品牌計費 vs 平台結算對平）</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>⬜〔標注 2026-07-22（Plane 對帳輪）：Plane 卡=In Pr</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr"/>
+      <c r="J14" s="8" t="inlineStr"/>
+      <c r="K14" s="8" t="inlineStr"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-24 ~ 2026-08-31</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>投影、對帳、intake 契約與第 2 品牌開站演練，M3 收斂</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>3.2.2</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>refinery intake 改走受控 API（ADR-042）：intake 端點 + DTO 資料最小化 + cursor/增量水位 + 逐租戶用量計量；REFINERY_POSTGRES_URI 直讀加 usage counter 後退場</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>ADR-042；ADR-036/040 憑證</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr"/>
+      <c r="J15" s="8" t="inlineStr"/>
+      <c r="K15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-24 ~ 2026-08-31</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>投影、對帳、intake 契約與第 2 品牌開站演練，M3 收斂</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>3.4.1</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>雲端拓撲對齊（tech / platform 面雲端部署 + 技師庫上雲）</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>⬜〔標注 2026-07-22（Plane 對帳輪）：Plane 卡=Done—</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>2.4.1</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr"/>
+      <c r="J16" s="8" t="inlineStr"/>
+      <c r="K16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-24 ~ 2026-08-31</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>投影、對帳、intake 契約與第 2 品牌開站演練，M3 收斂</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>3.5.1</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>第 2 品牌租戶開站演練（全流程 dry-run：申請 → 核准 → 開站 → 綁 LINE）</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>3.3.1</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr"/>
+      <c r="J17" s="8" t="inlineStr"/>
+      <c r="K17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>🛑 不排進衝刺 —— 待裁決，裁決下來才插隊</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>待裁決</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>混合派工（指派為主、搶單為輔）卡在 CR-0191 §8 的六項業主裁決。 沒裁決不能開工——搶單那一半是從零開始（現行只有候選 GIS 與評分排序， 師傅端無 accept/reject、offer 概念不存在），估不出工期也定不了驗收條件。</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>3.1.3</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>混合派工：指派為主、搶單為輔（指定師傅逾時未接 → 釋出公開池）。現行為純指派制，offer／accept／搶單併發控制全部不存在</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>🛑 待裁決</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>業主完成 CR-0191 §8 六項裁決後插入最近一個衝刺</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr"/>
+      <c r="J19" s="8" t="inlineStr"/>
+      <c r="K19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>⬜ 明確排除 —— M4：M4 平台化地基屬階段二（flow DSL 引擎、兩層渲染、Vertical Pack、積木庫、 FlowEditor、AI Onboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>不在本期範圍</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>刻意寫成一條宣告而不是「先不管它」——不指名的話，8 月底沒做完會被讀成滑期， 而它從一開始就不在範圍內。範圍砍掉是決定，不是失敗。</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>flow DSL 引擎產品化</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr"/>
+      <c r="J21" s="8" t="inlineStr"/>
+      <c r="K21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>不在本期範圍</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>刻意寫成一條宣告而不是「先不管它」——不指名的話，8 月底沒做完會被讀成滑期， 而它從一開始就不在範圍內。範圍砍掉是決定，不是失敗。</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>兩層渲染</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr"/>
+      <c r="J22" s="8" t="inlineStr"/>
+      <c r="K22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>不在本期範圍</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>刻意寫成一條宣告而不是「先不管它」——不指名的話，8 月底沒做完會被讀成滑期， 而它從一開始就不在範圍內。範圍砍掉是決定，不是失敗。</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Vertical Pack 打包</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr"/>
+      <c r="J23" s="8" t="inlineStr"/>
+      <c r="K23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>不在本期範圍</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>刻意寫成一條宣告而不是「先不管它」——不指名的話，8 月底沒做完會被讀成滑期， 而它從一開始就不在範圍內。範圍砍掉是決定，不是失敗。</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>積木庫 bootstrap</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr"/>
+      <c r="J24" s="8" t="inlineStr"/>
+      <c r="K24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>不在本期範圍</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>刻意寫成一條宣告而不是「先不管它」——不指名的話，8 月底沒做完會被讀成滑期， 而它從一開始就不在範圍內。範圍砍掉是決定，不是失敗。</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>FlowEditor 拖拉</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr"/>
+      <c r="J25" s="8" t="inlineStr"/>
+      <c r="K25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>不在本期範圍</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>刻意寫成一條宣告而不是「先不管它」——不指名的話，8 月底沒做完會被讀成滑期， 而它從一開始就不在範圍內。範圍砍掉是決定，不是失敗。</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>AI Onboarding Compiler</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr"/>
+      <c r="J26" s="8" t="inlineStr"/>
+      <c r="K26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>不在本期範圍</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>刻意寫成一條宣告而不是「先不管它」——不指名的話，8 月底沒做完會被讀成滑期， 而它從一開始就不在範圍內。範圍砍掉是決定，不是失敗。</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>第 2 產業落地</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr"/>
+      <c r="J27" s="8" t="inlineStr"/>
+      <c r="K27" s="8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K27"/>
+  <mergeCells count="2">
+    <mergeCell ref="A18:K18"/>
+    <mergeCell ref="A20:K20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>